<commit_message>
add API server + reorganize project + export excel+exportTable
</commit_message>
<xml_diff>
--- a/output/column_differences.xlsx
+++ b/output/column_differences.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
   <si>
     <t>Column Differences</t>
   </si>
@@ -26,19 +26,58 @@
     <t>Exists in</t>
   </si>
   <si>
-    <t>orders</t>
-  </si>
-  <si>
-    <t>order_date</t>
-  </si>
-  <si>
-    <t>db1 only</t>
-  </si>
-  <si>
-    <t>created_at</t>
-  </si>
-  <si>
-    <t>db2 only</t>
+    <t>country</t>
+  </si>
+  <si>
+    <t>numcode</t>
+  </si>
+  <si>
+    <t>d1 only</t>
+  </si>
+  <si>
+    <t>nicename</t>
+  </si>
+  <si>
+    <t>phonecode</t>
+  </si>
+  <si>
+    <t>iso3</t>
+  </si>
+  <si>
+    <t>department</t>
+  </si>
+  <si>
+    <t>location</t>
+  </si>
+  <si>
+    <t>d2 only</t>
+  </si>
+  <si>
+    <t>employee</t>
+  </si>
+  <si>
+    <t>date_of_probation_end</t>
+  </si>
+  <si>
+    <t>middle_names</t>
+  </si>
+  <si>
+    <t>date_of_termination</t>
+  </si>
+  <si>
+    <t>region</t>
+  </si>
+  <si>
+    <t>note</t>
+  </si>
+  <si>
+    <t>salary_group</t>
+  </si>
+  <si>
+    <t>base_salary</t>
+  </si>
+  <si>
+    <t>to_date</t>
   </si>
 </sst>
 </file>
@@ -160,11 +199,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="10.15234375" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="13.5859375" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="15.28125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="23.36328125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="13.11328125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -202,8 +241,118 @@
       <c r="B4" t="s" s="6">
         <v>7</v>
       </c>
-      <c r="C4" t="s" s="4">
+      <c r="C4" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s" s="5">
         <v>8</v>
+      </c>
+      <c r="C5" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="6">
+        <v>4</v>
+      </c>
+      <c r="B6" t="s" s="6">
+        <v>9</v>
+      </c>
+      <c r="C6" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="5">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s" s="5">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s" s="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="6">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s" s="6">
+        <v>14</v>
+      </c>
+      <c r="C8" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="5">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s" s="5">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="6">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s" s="6">
+        <v>16</v>
+      </c>
+      <c r="C10" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="5">
+        <v>17</v>
+      </c>
+      <c r="B11" t="s" s="5">
+        <v>18</v>
+      </c>
+      <c r="C11" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="6">
+        <v>17</v>
+      </c>
+      <c r="B12" t="s" s="6">
+        <v>7</v>
+      </c>
+      <c r="C12" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="5">
+        <v>19</v>
+      </c>
+      <c r="B13" t="s" s="5">
+        <v>20</v>
+      </c>
+      <c r="C13" t="s" s="3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="6">
+        <v>19</v>
+      </c>
+      <c r="B14" t="s" s="6">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s" s="3">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
build console-based database comparison engine (MySQL vs Oracle)
</commit_message>
<xml_diff>
--- a/output/column_differences.xlsx
+++ b/output/column_differences.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
   <si>
     <t>Column Differences</t>
   </si>
@@ -26,58 +26,25 @@
     <t>Exists in</t>
   </si>
   <si>
-    <t>country</t>
-  </si>
-  <si>
-    <t>numcode</t>
-  </si>
-  <si>
-    <t>d1 only</t>
-  </si>
-  <si>
-    <t>nicename</t>
-  </si>
-  <si>
-    <t>phonecode</t>
-  </si>
-  <si>
-    <t>iso3</t>
-  </si>
-  <si>
-    <t>department</t>
-  </si>
-  <si>
-    <t>location</t>
-  </si>
-  <si>
-    <t>d2 only</t>
-  </si>
-  <si>
-    <t>employee</t>
-  </si>
-  <si>
-    <t>date_of_probation_end</t>
-  </si>
-  <si>
-    <t>middle_names</t>
-  </si>
-  <si>
-    <t>date_of_termination</t>
-  </si>
-  <si>
-    <t>region</t>
-  </si>
-  <si>
-    <t>note</t>
-  </si>
-  <si>
-    <t>salary_group</t>
-  </si>
-  <si>
-    <t>base_salary</t>
-  </si>
-  <si>
-    <t>to_date</t>
+    <t>EMPLOYEES</t>
+  </si>
+  <si>
+    <t>NAME</t>
+  </si>
+  <si>
+    <t>XEPDB1 only</t>
+  </si>
+  <si>
+    <t>HIRE_DATE</t>
+  </si>
+  <si>
+    <t>FULL_NAME</t>
+  </si>
+  <si>
+    <t>DEPARTMENTS</t>
+  </si>
+  <si>
+    <t>LOCATION</t>
   </si>
 </sst>
 </file>
@@ -199,12 +166,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="15.28125" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="23.36328125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="13.11328125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="18.46484375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="15.4765625" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="16.26953125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1" ht="20.0" customHeight="true">
@@ -258,100 +225,12 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="6">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="B6" t="s" s="6">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C6" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s" s="5">
-        <v>10</v>
-      </c>
-      <c r="B7" t="s" s="5">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s" s="4">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s" s="6">
-        <v>13</v>
-      </c>
-      <c r="B8" t="s" s="6">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s" s="5">
-        <v>13</v>
-      </c>
-      <c r="B9" t="s" s="5">
-        <v>15</v>
-      </c>
-      <c r="C9" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s" s="6">
-        <v>13</v>
-      </c>
-      <c r="B10" t="s" s="6">
-        <v>16</v>
-      </c>
-      <c r="C10" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s" s="5">
-        <v>17</v>
-      </c>
-      <c r="B11" t="s" s="5">
-        <v>18</v>
-      </c>
-      <c r="C11" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s" s="6">
-        <v>17</v>
-      </c>
-      <c r="B12" t="s" s="6">
-        <v>7</v>
-      </c>
-      <c r="C12" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s" s="5">
-        <v>19</v>
-      </c>
-      <c r="B13" t="s" s="5">
-        <v>20</v>
-      </c>
-      <c r="C13" t="s" s="3">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s" s="6">
-        <v>19</v>
-      </c>
-      <c r="B14" t="s" s="6">
-        <v>21</v>
-      </c>
-      <c r="C14" t="s" s="3">
         <v>6</v>
       </c>
     </row>

</xml_diff>